<commit_message>
feat(F-NAR-009): 32 atomiques, ouvertures du monde distinctes
Détails d’abord (radiateur, clés, pluie, cacao…), puis l’action.
Troupe fermée. Texte seulement.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.002-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.002-01.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nora prend son manteau avant de sortir</t>
+          <t>Victorino et le manteau rouge</t>
         </is>
       </c>
     </row>
@@ -830,6 +830,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Victorino veut toucher les feuilles du jardin. Il prend le manteau rouge, sort avec maman, rentre, raccroche.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1184,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Nora est près de la porte. Maman lace ses chaussures. On va au jardin. Avant de sortir, Nora prend son manteau. Le manteau est rouge. Il est un peu épais. Nora glisse un bras. Nora glisse l'autre bras. Le manteau est chaud. Nora et maman vont au jardin. L'air est frais. Nora touche une feuille. La feuille est lisse. C'est l'heure de rentrer. Elles vont rentrer. Nora entre dans la maison. Nora retire le manteau. Elle le raccroche au crochet. Le crochet est bas. Le manteau est à sa place. Merci Nora.</t>
+          <t>Le radiateur fait tic tic tic. Des chaussettes sèchent dessus. Elles sont épaisses et douces. Une lumière jaune touche le carrelage. La maison sent le linge chaud. Victorino, tu viens près de la porte ? Derrière la vitre, le jardin est pâle. Une feuille collée tremble un peu. En ce moment, Victorino est dans le hall. Son manteau rouge attend au crochet. Le crochet est bas. Il est à sa hauteur. Maman, on va au jardin ? Oui. On va au jardin. Avant de sortir, on prend le manteau. Victorino touche le manteau. Le tissu est un peu épais. Il est rouge comme une pomme. Il est chaud. Oui. Il te tiendra chaud. Glisse un bras. Victorino glisse un bras. Maintenant l'autre bras. Victorino glisse l'autre bras. Bravo. Tu as pris ton manteau. Maman lace les chaussures. Les lacets font un petit bruit. Tu es prêt ? Oui. On sort. Maman ouvre la porte. L'air est frais. Ça sent la terre. Ils vont au jardin. Victorino marche près de maman. Il touche une feuille. La feuille est lisse. Elle est un peu froide. Elle est mouillée, maman. Oui. La feuille a de l'eau. Tu as les mains au chaud ? Oui. Dans les poches. Ils restent un petit moment. Un oiseau passe tout bas. Tu as vu l'oiseau ? Oui. Il est parti. C'est l'heure de rentrer. Ils rentrent dans la maison. La maison est tiède. En rentrant, on pose le manteau. Victorino retire le manteau. Il le raccroche au crochet. Le crochet est bas. Le manteau rouge est à sa place. Bravo, Victorino. Tu as fait du bon travail. Le manteau est au crochet ? Oui. Il est là.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,15 +1324,70 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Nora est près de la porte. Maman lace ses chaussures.
-maman|On va au jardin. Avant de sortir, Nora prend son manteau.
-narrateur|Le manteau est rouge. Il est un peu épais. Nora glisse un bras. Nora glisse l'autre bras. Le manteau est chaud. Nora et maman vont au jardin. L'air est frais. Nora touche une feuille. La feuille est lisse.
-maman|C'est l'heure de rentrer. Elles vont rentrer.
-narrateur|Nora entre dans la maison. Nora retire le manteau. Elle le raccroche au crochet. Le crochet est bas. Le manteau est à sa place.
-maman|Merci Nora.</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr"/>
+          <t>narrateur|Le radiateur fait tic tic tic.
+narrateur|Des chaussettes sèchent dessus.
+narrateur|Elles sont épaisses et douces.
+narrateur|Une lumière jaune touche le carrelage.
+narrateur|La maison sent le linge chaud.
+maman|Victorino, tu viens près de la porte ?
+narrateur|Derrière la vitre, le jardin est pâle.
+narrateur|Une feuille collée tremble un peu.
+narrateur|En ce moment, Victorino est dans le hall.
+narrateur|Son manteau rouge attend au crochet.
+narrateur|Le crochet est bas.
+narrateur|Il est à sa hauteur.
+enfant-m|Maman, on va au jardin ?
+maman|Oui. On va au jardin.
+maman|Avant de sortir, on prend le manteau.
+narrateur|Victorino touche le manteau.
+narrateur|Le tissu est un peu épais.
+narrateur|Il est rouge comme une pomme.
+enfant-m|Il est chaud.
+maman|Oui. Il te tiendra chaud.
+maman|Glisse un bras.
+narrateur|Victorino glisse un bras.
+maman|Maintenant l'autre bras.
+narrateur|Victorino glisse l'autre bras.
+maman|Bravo. Tu as pris ton manteau.
+narrateur|Maman lace les chaussures.
+narrateur|Les lacets font un petit bruit.
+maman|Tu es prêt ?
+enfant-m|Oui. On sort.
+narrateur|Maman ouvre la porte.
+narrateur|L'air est frais.
+narrateur|Ça sent la terre.
+narrateur|Ils vont au jardin.
+narrateur|Victorino marche près de maman.
+narrateur|Il touche une feuille.
+narrateur|La feuille est lisse.
+narrateur|Elle est un peu froide.
+enfant-m|Elle est mouillée, maman.
+maman|Oui. La feuille a de l'eau.
+maman|Tu as les mains au chaud ?
+enfant-m|Oui. Dans les poches.
+narrateur|Ils restent un petit moment.
+narrateur|Un oiseau passe tout bas.
+maman|Tu as vu l'oiseau ?
+enfant-m|Oui. Il est parti.
+maman|C'est l'heure de rentrer.
+narrateur|Ils rentrent dans la maison.
+narrateur|La maison est tiède.
+maman|En rentrant, on pose le manteau.
+narrateur|Victorino retire le manteau.
+narrateur|Il le raccroche au crochet.
+narrateur|Le crochet est bas.
+narrateur|Le manteau rouge est à sa place.
+maman|Bravo, Victorino.
+maman|Tu as fait du bon travail.
+maman|Le manteau est au crochet ?
+enfant-m|Oui. Il est là.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>radiateur,porte</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1345,7 +1412,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Nora ?</t>
+          <t>Avant de sortir, que prend Victorino ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1505,7 +1572,7 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de sortir, que prend Nora ?</t>
+          <t>narrateur|Avant de sortir, que prend Victorino ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1533,7 +1600,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nora a pris le manteau. Elle est sortie. En rentrant, elle l'a raccroché. Le manteau est à sa place.</t>
+          <t>Victorino a pris le manteau. Le manteau rouge. Il est sorti au jardin. Il a touché une feuille. En rentrant, il l'a raccroché. Le manteau est à sa place. Bravo. Tu as pris le manteau. Et tu l'as raccroché. C'est du bon travail. Il est au crochet, maman. Oui. Il attend pour la prochaine fois.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1677,7 +1744,17 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nora a pris le manteau. Elle est sortie. En rentrant, elle l'a raccroché. Le manteau est à sa place.</t>
+          <t>narrateur|Victorino a pris le manteau.
+narrateur|Le manteau rouge.
+narrateur|Il est sorti au jardin.
+narrateur|Il a touché une feuille.
+narrateur|En rentrant, il l'a raccroché.
+narrateur|Le manteau est à sa place.
+maman|Bravo. Tu as pris le manteau.
+maman|Et tu l'as raccroché.
+maman|C'est du bon travail.
+enfant-m|Il est au crochet, maman.
+maman|Oui. Il attend pour la prochaine fois.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1705,7 +1782,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nora pose les chaussures. Le manteau reste au crochet. Maman sourit.</t>
+          <t>Victorino pose les chaussures. Elles restent près de la porte. Les chaussettes sont encore tièdes. Tu as les pieds au chaud ? Oui, maman. Le manteau rouge reste au crochet. Le hall est calme. Le radiateur fait encore tic tic. On reste un peu à la maison ? Oui. Un peu. Bravo. Tu as bien fait.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1845,7 +1922,17 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nora pose les chaussures. Le manteau reste au crochet. Maman sourit.</t>
+          <t>narrateur|Victorino pose les chaussures.
+narrateur|Elles restent près de la porte.
+narrateur|Les chaussettes sont encore tièdes.
+maman|Tu as les pieds au chaud ?
+enfant-m|Oui, maman.
+narrateur|Le manteau rouge reste au crochet.
+narrateur|Le hall est calme.
+narrateur|Le radiateur fait encore tic tic.
+maman|On reste un peu à la maison ?
+enfant-m|Oui. Un peu.
+maman|Bravo. Tu as bien fait.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1873,7 +1960,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>J'ai pris le manteau. Je l'ai raccroché. Bravo, Victorino. Tu as fait du bon travail. Le jardin est derrière la vitre. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2013,7 +2100,12 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>enfant-m|J'ai pris le manteau.
+enfant-m|Je l'ai raccroché.
+maman|Bravo, Victorino.
+maman|Tu as fait du bon travail.
+narrateur|Le jardin est derrière la vitre.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2035,7 +2127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2073,6 +2165,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(F-NAR-008): retirer les refrains de leçon du catalogue réécrit
Plus de « tu as fait du bon travail », « L'histoire est finie »,
ni de récap « tu as mis ce que l'adulte a dit ». Fin = image vécue.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.002-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.002-01.xlsx
@@ -1969,12 +1969,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai mis la feuille dans le bol. J'avais le manteau. Bravo, Victorino. Tu as fait du bon travail. Le bol blanc brille encore. L'histoire est finie.</t>
+          <t>J'ai mis la feuille dans le bol. J'avais le manteau. Bravo, Victorino. Le bol blanc brille encore.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai mis la feuille dans le bol. J'avais le manteau. Bravo, Victorino. Tu as fait du bon travail. Le bol blanc brille encore. L'histoire est finie.</t>
+          <t>J'ai mis la feuille dans le bol. J'avais le manteau. Bravo, Victorino. Le bol blanc brille encore.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2112,9 +2112,7 @@
           <t>enfant-m|J'ai mis la feuille dans le bol.
 enfant-m|J'avais le manteau.
 maman|Bravo, Victorino.
-maman|Tu as fait du bon travail.
-narrateur|Le bol blanc brille encore.
-narrateur|L'histoire est finie.</t>
+narrateur|Le bol blanc brille encore.</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2220,6 +2218,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
fix(F-NAR-008): troupe D16 aussi dans la fiche (plus de Nora/Lina)
apply écrit characters et setting. 659 ATOM alignés sur merged.json.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.002-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.002-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison et jardin</t>
+          <t>maison et jardin, vitre mouillée</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nora, maman</t>
+          <t>Victorino, maman</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.002-01 La feuille rouge de Victorino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.002-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.002-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison et jardin, vitre mouillée</t>
+          <t>maison et jardin, vitre mouillée, sentier d'eau</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino veut la feuille rouge collée à la vitre, pour le bol blanc. Une manche du manteau est à l'envers. Maman tourne le tissu. Ils ramassent la feuille. Le manteau rentre au crochet. La feuille brille dans le bol.</t>
+          <t>La pluie écrit sur la vitre. Un trait de vitre descend, fin. Victorino veut la feuille rouge maintenant, pour le bol. Il tire le manteau : la manche reste à l'envers. Il refuse de foncer, dit qu'il le met, tourne la manche. Au jardin, la feuille glisse. Il suit le trait de vitre. Dans le bol, le trait brille sur la feuille.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une goutte glisse sur la vitre. Elle laisse un trait brillant. Une feuille rouge est collée. On dirait une petite étoile. La cuisine sent le pain tiède. Maman essuie la table en bois. Un bol blanc attend au milieu. La lumière est jaune et douce. Victorino vit ici, avec maman. Maman, la feuille est rouge ! Oui. Elle est collée à la vitre. En ce moment, Victorino s'approche. Il pose le doigt sur le verre. Le verre est un peu froid. Je la veux pour le bol. On peut aller la chercher. Elle est tombée dans le jardin. Victorino court vers la porte. Le manteau rouge attend au crochet. Le crochet est bas, à sa hauteur. Il tire le manteau vers lui. Une manche est à l'envers. Son bras ne passe pas. Oh. Je n'y arrive pas. Attends. On tourne la manche. Maman tourne le tissu tout doux. Le rouge est chaud comme une pomme. Glisse un bras. Victorino glisse un bras. Maintenant l'autre. Victorino glisse l'autre bras. Il est chaud. Oui. Il te tiendra chaud dehors. On ouvre la porte ? Oui. On va chercher la feuille. Maman ouvre la porte. L'air sent la terre mouillée. Le jardin est pâle et calme. Victorino marche près de maman. L'herbe est un peu froide. La feuille rouge est dans l'herbe. Elle est là ! Tu la prends tout doux ? Victorino ramasse la feuille. Elle est lisse et un peu mouillée. Il la glisse dans la poche. Elle est dans la poche. Bien. Tes mains sont au chaud ? Oui. Dans les poches. Un oiseau passe tout bas. Tu as vu l'oiseau ? Oui. Il est parti. C'est l'heure de rentrer. Ils rentrent dans la maison. La maison est tiède. Victorino retire le manteau rouge. Il le raccroche au crochet. Le manteau est à sa place. Je sors la feuille. Il prend la feuille dans la poche. Il la pose dans le bol blanc. Elle est belle, dans le bol. C'est ma feuille rouge. Oui.</t>
+          <t>La pluie écrit sur la vitre. Elle trace une ligne brillante. Un trait de vitre descend, fin. Derrière, une feuille rouge est collée. Maman, elle est rouge ! Oui. Elle est collée au verre. La cuisine sent le pain tiède. Sur la table, un bol blanc attend. Le bois de la table est lisse. Une odeur de pain reste dans l'air. Un carré de lumière touche le bol. Le bol est vide, et rond. Victorino lève les yeux vers la vitre. La vitre est mouillée, un peu froide. On dirait une petite étoile. Maman essuie le rebord, sans presser. En ce moment, Victorino s'approche. Il pose le doigt sur le verre. Le verre pique un peu, froid. Son souffle fait un nuage rond. Il essuie le nuage du pouce. Je la veux maintenant, pour le bol. Tu la veux vite ? Oui, maman. Elle est tombée, dans le jardin. On peut aller la chercher. Victorino court vers la porte. Son pied tape le carreau, impatient. La porte de bois est close. Le manteau rouge attend au crochet. Le crochet est bas, à sa hauteur. Le tissu est épais, un peu rêche. Il tire le manteau d'un coup. Une manche est à l'envers. Son bras ne passe pas. Oh. Ça ne veut pas. Le manteau tombe un peu, lourd. Ses épaules tombent un peu. Ça serre, dans son ventre. Le sourire quitte sa bouche. Maman se baisse à sa hauteur. Tu regardes la manche ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une goutte glisse sur la vitre. Elle laisse un trait brillant. Une feuille rouge est collée. On dirait une petite étoile. La cuisine sent le pain tiède. Maman essuie la table en bois. Un bol blanc attend au milieu. La lumière est jaune et douce. Victorino vit ici, avec maman. Maman, la feuille est rouge ! Oui. Elle est collée à la vitre. En ce moment, Victorino s'approche. Il pose le doigt sur le verre. Le verre est un peu froid. Je la veux pour le bol. On peut aller la chercher. Elle est tombée dans le jardin. Victorino court vers la porte. Le manteau rouge attend au crochet. Le crochet est bas, à sa hauteur. Il tire le manteau vers lui. Une manche est à l'envers. Son bras ne passe pas. Oh. Je n'y arrive pas. Attends. On tourne la manche. Maman tourne le tissu tout doux. Le rouge est chaud comme une pomme. Glisse un bras. Victorino glisse un bras. Maintenant l'autre. Victorino glisse l'autre bras. Il est chaud. Oui. Il te tiendra chaud dehors. On ouvre la porte ? Oui. On va chercher la feuille. Maman ouvre la porte. L'air sent la terre mouillée. Le jardin est pâle et calme. Victorino marche près de maman. L'herbe est un peu froide. La feuille rouge est dans l'herbe. Elle est là ! Tu la prends tout doux ? Victorino ramasse la feuille. Elle est lisse et un peu mouillée. Il la glisse dans la poche. Elle est dans la poche. Bien. Tes mains sont au chaud ? Oui. Dans les poches. Un oiseau passe tout bas. Tu as vu l'oiseau ? Oui. Il est parti. C'est l'heure de rentrer. Ils rentrent dans la maison. La maison est tiède. Victorino retire le manteau rouge. Il le raccroche au crochet. Le manteau est à sa place. Je sors la feuille. Il prend la feuille dans la poche. Il la pose dans le bol blanc. Elle est belle, dans le bol. C'est ma feuille rouge. Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pluie écrit sur la vitre. Elle trace une ligne brillante. Un &lt;emphasis level="moderate"&gt;trait de vitre&lt;/emphasis&gt; descend, fin. Derrière, une feuille rouge est collée. Maman, elle est rouge ! Oui. Elle est collée au verre. La cuisine sent le pain tiède. Sur la table, un bol blanc attend. Le bois de la table est lisse. Une odeur de pain reste dans l'air. Un carré de lumière touche le bol. Le bol est vide, et rond. Victorino lève les yeux vers la vitre. La vitre est mouillée, un peu froide. On dirait une petite étoile. Maman essuie le rebord, sans presser. En ce moment, Victorino s'approche. Il pose le doigt sur le verre. Le verre pique un peu, froid. Son souffle fait un nuage rond. Il essuie le nuage du pouce. Je la veux maintenant, pour le bol. Tu la veux vite ? Oui, maman. Elle est tombée, dans le jardin. On peut aller la chercher. Victorino court vers la porte. Son pied tape le carreau, impatient. La porte de bois est close. Le manteau rouge attend au crochet. Le crochet est bas, à sa hauteur. Le tissu est épais, un peu rêche. Il tire le manteau d'un coup. Une manche est à l'envers. Son bras ne passe pas. Oh. Ça ne veut pas. Le manteau tombe un peu, lourd. Ses épaules tombent un peu. Ça serre, dans son ventre. Le sourire quitte sa bouche. Maman se baisse à sa hauteur. Tu regardes la manche ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Nora est près de la porte. Maman lace ses chaussures. Maman dit : on va au jardin. Avant de sortir, Nora prend son &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Le manteau est rouge. Il est un peu épais. Nora glisse un bras. Nora glisse l'autre bras. Le manteau est chaud. Nora et maman vont au jardin. L'air est frais. Nora touche une feuille. La feuille est lisse. Maman dit : c'est l'heure de rentrer. Elles vont rentrer. Nora entre dans la maison. Nora retire le manteau. Elle le raccroche au crochet. Le crochet est bas. Le manteau est à sa place. Maman dit : merci Nora.&lt;/slow&gt; [pause]</t>
+          <t>La pluie écrit sur la vitre. Elle trace une ligne brillante. Un &lt;emphasis&gt;trait de vitre&lt;/emphasis&gt; descend, fin. Derrière, une feuille rouge est collée. Maman, elle est rouge ! Oui. Elle est collée au verre. La cuisine sent le pain tiède. Sur la table, un bol blanc attend. Le bois de la table est lisse. Une odeur de pain reste dans l'air. Un carré de lumière touche le bol. Le bol est vide, et rond. Victorino lève les yeux vers la vitre. La vitre est mouillée, un peu froide. On dirait une petite étoile. Maman essuie le rebord, sans presser. En ce moment, Victorino s'approche. Il pose le doigt sur le verre. Le verre pique un peu, froid. Son souffle fait un nuage rond. Il essuie le nuage du pouce. Je la veux maintenant, pour le bol. Tu la veux vite ? Oui, maman. Elle est tombée, dans le jardin. On peut aller la chercher. Victorino court vers la porte. Son pied tape le carreau, impatient. La porte de bois est close. Le manteau rouge attend au crochet. Le crochet est bas, à sa hauteur. Le tissu est épais, un peu rêche. Il tire le manteau d'un coup. Une manche est à l'envers. Son bras ne passe pas. Oh. Ça ne veut pas. Le manteau tombe un peu, lourd. Ses épaules tombent un peu. Ça serre, dans son ventre. Le sourire quitte sa bouche. Maman se baisse à sa hauteur. Tu regardes la manche ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>trait de vitre</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,88 +1319,64 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_feuille_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une goutte glisse sur la vitre.
-narrateur|Elle laisse un trait brillant.
-narrateur|Une feuille rouge est collée.
+          <t>narrateur|La pluie écrit sur la vitre.
+narrateur|Elle trace une ligne brillante.
+narrateur|Un trait de vitre descend, fin.
+narrateur|Derrière, une feuille rouge est collée.
+enfant-m|Maman, elle est rouge !
+maman|Oui.
+maman|Elle est collée au verre.
+narrateur|La cuisine sent le pain tiède.
+narrateur|Sur la table, un bol blanc attend.
+narrateur|Le bois de la table est lisse.
+narrateur|Une odeur de pain reste dans l'air.
+narrateur|Un carré de lumière touche le bol.
+narrateur|Le bol est vide, et rond.
+narrateur|Victorino lève les yeux vers la vitre.
+narrateur|La vitre est mouillée, un peu froide.
 narrateur|On dirait une petite étoile.
-narrateur|La cuisine sent le pain tiède.
-narrateur|Maman essuie la table en bois.
-narrateur|Un bol blanc attend au milieu.
-narrateur|La lumière est jaune et douce.
-narrateur|Victorino vit ici, avec maman.
-enfant-m|Maman, la feuille est rouge !
-maman|Oui.
-maman|Elle est collée à la vitre.
+narrateur|Maman essuie le rebord, sans presser.
 narrateur|En ce moment, Victorino s'approche.
 narrateur|Il pose le doigt sur le verre.
-narrateur|Le verre est un peu froid.
-enfant-m|Je la veux pour le bol.
+narrateur|Le verre pique un peu, froid.
+narrateur|Son souffle fait un nuage rond.
+narrateur|Il essuie le nuage du pouce.
+enfant-m|Je la veux maintenant, pour le bol.
+maman|Tu la veux vite ?
+enfant-m|Oui, maman.
+maman|Elle est tombée, dans le jardin.
 maman|On peut aller la chercher.
-maman|Elle est tombée dans le jardin.
 narrateur|Victorino court vers la porte.
+narrateur|Son pied tape le carreau, impatient.
+narrateur|La porte de bois est close.
 narrateur|Le manteau rouge attend au crochet.
 narrateur|Le crochet est bas, à sa hauteur.
-narrateur|Il tire le manteau vers lui.
+narrateur|Le tissu est épais, un peu rêche.
+narrateur|Il tire le manteau d'un coup.
 narrateur|Une manche est à l'envers.
 narrateur|Son bras ne passe pas.
 enfant-m|Oh.
-enfant-m|Je n'y arrive pas.
-maman|Attends.
-maman|On tourne la manche.
-narrateur|Maman tourne le tissu tout doux.
-narrateur|Le rouge est chaud comme une pomme.
-maman|Glisse un bras.
-narrateur|Victorino glisse un bras.
-maman|Maintenant l'autre.
-narrateur|Victorino glisse l'autre bras.
-enfant-m|Il est chaud.
-maman|Oui.
-maman|Il te tiendra chaud dehors.
-maman|On ouvre la porte ?
-enfant-m|Oui.
-enfant-m|On va chercher la feuille.
-narrateur|Maman ouvre la porte.
-narrateur|L'air sent la terre mouillée.
-narrateur|Le jardin est pâle et calme.
-narrateur|Victorino marche près de maman.
-narrateur|L'herbe est un peu froide.
-narrateur|La feuille rouge est dans l'herbe.
-enfant-m|Elle est là !
-maman|Tu la prends tout doux ?
-narrateur|Victorino ramasse la feuille.
-narrateur|Elle est lisse et un peu mouillée.
-narrateur|Il la glisse dans la poche.
-enfant-m|Elle est dans la poche.
-maman|Bien.
-maman|Tes mains sont au chaud ?
-enfant-m|Oui.
-enfant-m|Dans les poches.
-narrateur|Un oiseau passe tout bas.
-maman|Tu as vu l'oiseau ?
-enfant-m|Oui.
-enfant-m|Il est parti.
-maman|C'est l'heure de rentrer.
-narrateur|Ils rentrent dans la maison.
-narrateur|La maison est tiède.
-narrateur|Victorino retire le manteau rouge.
-narrateur|Il le raccroche au crochet.
-narrateur|Le manteau est à sa place.
-enfant-m|Je sors la feuille.
-narrateur|Il prend la feuille dans la poche.
-narrateur|Il la pose dans le bol blanc.
-maman|Elle est belle, dans le bol.
-enfant-m|C'est ma feuille rouge.
-maman|Oui.</t>
+enfant-m|Ça ne veut pas.
+narrateur|Le manteau tombe un peu, lourd.
+narrateur|Ses épaules tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Le sourire quitte sa bouche.
+narrateur|Maman se baisse à sa hauteur.
+maman|Tu regardes la manche ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>porte</t>
+          <t>pluie,vitre,porte</t>
         </is>
       </c>
     </row>
@@ -1427,17 +1403,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Victorino ?</t>
+          <t>Victorino veut sortir. Que prend-il, avant la porte ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Victorino ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino veut &lt;emphasis level="moderate"&gt;sortir&lt;/emphasis&gt;. Que prend-il, avant la porte ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Avant de &lt;emphasis&gt;sortir&lt;/emphasis&gt;, que prend Nora ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorino veut &lt;emphasis&gt;sortir&lt;/emphasis&gt;. Que prend-il, avant la porte ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1500,7 +1476,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1508,10 +1484,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1526,11 +1502,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1541,23 +1517,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1566,13 +1542,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1582,12 +1558,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_prend_le_manteau; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de sortir, que prend Victorino ?</t>
+          <t>narrateur|Victorino veut sortir.
+narrateur|Que prend-il, avant la porte ?</t>
         </is>
       </c>
     </row>
@@ -1614,17 +1591,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorino a pris le manteau rouge. Il est allé au jardin. Il a ramassé la feuille. En rentrant, il a raccroché. La feuille est dans le bol. Tu as pris le manteau pour sortir. Il est au crochet, maman. Oui. Il attend pour la prochaine fois.</t>
+          <t>Je prends le manteau. Victorino refuse de tirer plus fort. Il pose un genou au sol. La manche est plate, tournée. Je la tourne, moi. Il retourne le tissu, lentement. La manche s'ouvre, large. Elle est libre. Il veut courir vers la porte. Le second bras reste coincé. Oh. Il ne tire pas trop vite. Il écoute le tissu, un instant. Il glisse un bras, puis l'autre. Le rouge est chaud comme une pomme. Il est chaud. Je le mets, moi. Oui. Il te tiendra chaud dehors. Tu fermes le bouton ? Victorino pousse le bouton, un clic. Le manteau rouge est fermé. Le col touche sa joue, chaud. Merci, Victorino. Victorino pose la main sur le tissu. Le tissu est un peu rêche. Le manteau est prêt ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorino a pris le manteau rouge. Il est allé au jardin. Il a ramassé la feuille. En rentrant, il a raccroché. La feuille est dans le bol. Tu as pris le manteau pour sortir. Il est au crochet, maman. Oui. Il attend pour la prochaine fois.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je prends le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt;. Victorino refuse de tirer plus fort. Il pose un genou au sol. La manche est plate, tournée. Je la tourne, moi. Il retourne le tissu, lentement. La manche s'ouvre, large. Elle est libre. Il veut courir vers la porte. Le second bras reste coincé. Oh. Il ne tire pas trop vite. Il écoute le tissu, un instant. Il glisse un bras, puis l'autre. Le rouge est chaud comme une pomme. Il est chaud. Je le mets, moi. Oui. Il te tiendra chaud dehors. Tu fermes le bouton ? Victorino pousse le bouton, un clic. Le manteau rouge est fermé. Le col touche sa joue, chaud. Merci, Victorino. Victorino pose la main sur le tissu. Le tissu est un peu rêche. Le manteau est prêt ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Nora a pris le &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Elle est sortie. En rentrant, elle l'a raccroché. Le manteau est à sa place.&lt;/slow&gt; [pause]</t>
+          <t>Je prends le &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Victorino refuse de tirer plus fort. Il pose un genou au sol. La manche est plate, tournée. Je la tourne, moi. Il retourne le tissu, lentement. La manche s'ouvre, large. Elle est libre. Il veut courir vers la porte. Le second bras reste coincé. Oh. Il ne tire pas trop vite. Il écoute le tissu, un instant. Il glisse un bras, puis l'autre. Le rouge est chaud comme une pomme. Il est chaud. Je le mets, moi. Oui. Il te tiendra chaud dehors. Tu fermes le bouton ? Victorino pousse le bouton, un clic. Le manteau rouge est fermé. Le col touche sa joue, chaud. Merci, Victorino. Victorino pose la main sur le tissu. Le tissu est un peu rêche. Le manteau est prêt ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1671,18 +1648,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1712,23 +1689,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1737,10 +1714,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1749,24 +1726,48 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_dit_et_met_le_manteau; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorino a pris le manteau rouge.
-narrateur|Il est allé au jardin.
-narrateur|Il a ramassé la feuille.
-narrateur|En rentrant, il a raccroché.
-narrateur|La feuille est dans le bol.
-maman|Tu as pris le manteau pour sortir.
-enfant-m|Il est au crochet, maman.
+          <t>enfant-m|Je prends le manteau.
+narrateur|Victorino refuse de tirer plus fort.
+narrateur|Il pose un genou au sol.
+narrateur|La manche est plate, tournée.
+enfant-m|Je la tourne, moi.
+narrateur|Il retourne le tissu, lentement.
+narrateur|La manche s'ouvre, large.
+enfant-m|Elle est libre.
+narrateur|Il veut courir vers la porte.
+narrateur|Le second bras reste coincé.
+enfant-m|Oh.
+narrateur|Il ne tire pas trop vite.
+narrateur|Il écoute le tissu, un instant.
+narrateur|Il glisse un bras, puis l'autre.
+narrateur|Le rouge est chaud comme une pomme.
+enfant-m|Il est chaud.
+enfant-m|Je le mets, moi.
 maman|Oui.
-maman|Il attend pour la prochaine fois.</t>
+maman|Il te tiendra chaud dehors.
+maman|Tu fermes le bouton ?
+narrateur|Victorino pousse le bouton, un clic.
+narrateur|Le manteau rouge est fermé.
+narrateur|Le col touche sa joue, chaud.
+maman|Merci, Victorino.
+narrateur|Victorino pose la main sur le tissu.
+narrateur|Le tissu est un peu rêche.
+maman|Le manteau est prêt ?
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>manteau,bouton</t>
         </is>
       </c>
     </row>
@@ -1793,17 +1794,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Victorino pose les chaussures. Elles restent près de la porte. Le bol blanc brille un peu. Tu as les pieds au chaud ? Oui, maman. Le manteau rouge reste au crochet. La vitre n'a plus de feuille. On reste un peu à la maison ? Oui. Avec ma feuille.</t>
+          <t>On met tes chaussures ? Victorino enfile ses chaussures. Une semelle est froide. Tu as fini tes chaussures ? Oui, maman. On ouvre la porte ? Oui. On va chercher la feuille. Maman ouvre la porte. L'air sent la terre mouillée. Le jardin est pâle, luisant. Un sentier d'eau coupe l'herbe. Victorino marche près de maman. L'herbe est un peu froide. Je la vois ! La feuille rouge brille dans l'herbe. Il tend la main, trop vite. La feuille glisse sous l'herbe. Elle part ! Victorino recule d'un pas. Il refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. L'envie et l'inquiétude se bousculent. Personne ne dit la suite. Il lève les yeux vers la vitre. Le trait de vitre brille, dehors. Il pointe vers l'herbe. Tu le suis, ce trait ? Oui. Il suit le trait, sans courir. Au pied du mur, l'herbe s'ouvre. La feuille rouge est là. Te voilà. Tu la prends sans presser ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Victorino pose les chaussures. Elles restent près de la porte. Le bol blanc brille un peu. Tu as les pieds au chaud ? Oui, maman. Le manteau rouge reste au crochet. La vitre n'a plus de feuille. On reste un peu à la maison ? Oui. Avec ma feuille.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On met tes chaussures ? Victorino enfile ses chaussures. Une semelle est froide. Tu as fini tes chaussures ? Oui, maman. On ouvre la porte ? Oui. On va chercher la &lt;emphasis level="moderate"&gt;feuille&lt;/emphasis&gt;. Maman ouvre la porte. L'air sent la terre mouillée. Le jardin est pâle, luisant. Un sentier d'eau coupe l'herbe. Victorino marche près de maman. L'herbe est un peu froide. Je la vois ! La feuille rouge brille dans l'herbe. Il tend la main, trop vite. La feuille glisse sous l'herbe. Elle part ! Victorino recule d'un pas. Il refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. L'envie et l'inquiétude se bousculent. Personne ne dit la suite. Il lève les yeux vers la vitre. Le trait de vitre brille, dehors. Il pointe vers l'herbe. Tu le suis, ce trait ? Oui. Il suit le trait, sans courir. Au pied du mur, l'herbe s'ouvre. La feuille rouge est là. Te voilà. Tu la prends sans presser ? Oui, maman.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Nora pose les chaussures. Le &lt;emphasis&gt;manteau&lt;/emphasis&gt; reste au crochet. Maman sourit.&lt;/slow&gt; [pause]</t>
+          <t>On met tes chaussures ? Victorino enfile ses chaussures. Une semelle est froide. Tu as fini tes chaussures ? Oui, maman. On ouvre la porte ? Oui. On va chercher la &lt;emphasis&gt;feuille&lt;/emphasis&gt;. Maman ouvre la porte. L'air sent la terre mouillée. Le jardin est pâle, luisant. Un sentier d'eau coupe l'herbe. Victorino marche près de maman. L'herbe est un peu froide. Je la vois ! La feuille rouge brille dans l'herbe. Il tend la main, trop vite. La feuille glisse sous l'herbe. Elle part ! Victorino recule d'un pas. Il refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. L'envie et l'inquiétude se bousculent. Personne ne dit la suite. Il lève les yeux vers la vitre. Le trait de vitre brille, dehors. Il pointe vers l'herbe. Tu le suis, ce trait ? Oui. Il suit le trait, sans courir. Au pied du mur, l'herbe s'ouvre. La feuille rouge est là. Te voilà. Tu la prends sans presser ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1850,18 +1851,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1884,30 +1885,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>feuille</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1916,10 +1917,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1928,21 +1929,56 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Victorino pose les chaussures.
-narrateur|Elles restent près de la porte.
-narrateur|Le bol blanc brille un peu.
-maman|Tu as les pieds au chaud ?
+          <t>maman|On met tes chaussures ?
+narrateur|Victorino enfile ses chaussures.
+narrateur|Une semelle est froide.
+maman|Tu as fini tes chaussures ?
 enfant-m|Oui, maman.
-narrateur|Le manteau rouge reste au crochet.
-narrateur|La vitre n'a plus de feuille.
-maman|On reste un peu à la maison ?
+maman|On ouvre la porte ?
 enfant-m|Oui.
-enfant-m|Avec ma feuille.</t>
+enfant-m|On va chercher la feuille.
+narrateur|Maman ouvre la porte.
+narrateur|L'air sent la terre mouillée.
+narrateur|Le jardin est pâle, luisant.
+narrateur|Un sentier d'eau coupe l'herbe.
+narrateur|Victorino marche près de maman.
+narrateur|L'herbe est un peu froide.
+enfant-m|Je la vois !
+narrateur|La feuille rouge brille dans l'herbe.
+narrateur|Il tend la main, trop vite.
+narrateur|La feuille glisse sous l'herbe.
+enfant-m|Elle part !
+narrateur|Victorino recule d'un pas.
+narrateur|Il refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|L'envie et l'inquiétude se bousculent.
+narrateur|Personne ne dit la suite.
+narrateur|Il lève les yeux vers la vitre.
+narrateur|Le trait de vitre brille, dehors.
+enfant-m|Il pointe vers l'herbe.
+maman|Tu le suis, ce trait ?
+enfant-m|Oui.
+narrateur|Il suit le trait, sans courir.
+narrateur|Au pied du mur, l'herbe s'ouvre.
+narrateur|La feuille rouge est là.
+enfant-m|Te voilà.
+maman|Tu la prends sans presser ?
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>porte,jardin</t>
         </is>
       </c>
     </row>
@@ -1969,17 +2005,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai mis la feuille dans le bol. J'avais le manteau. Bravo, Victorino. Le bol blanc brille encore.</t>
+          <t>Victorino ramasse la feuille, sans presser. Elle est lisse, un peu mouillée. Il la glisse dans la poche. Elle est dans la poche. Tes mains sont au chaud ? Oui. Dans les poches. Ils rentrent dans la maison. La maison est tiède. La chaleur touche les joues de Victorino. Victorino retire le manteau rouge. Il le raccroche au crochet. Le crochet fait un petit bruit. Le manteau est à sa place. Je sors la feuille. Il prend la feuille dans la poche. Il la pose dans le bol blanc. Comme sur la vitre, maman ! Sur la feuille, un trait brille. Le trait de vitre est sur la feuille. Tu le vois, sur ta feuille ? Oui. C'est ma feuille rouge. Le bol blanc garde la feuille. Le trait de vitre dore, mince.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai mis la feuille dans le bol. J'avais le manteau. Bravo, Victorino. Le bol blanc brille encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Victorino ramasse la feuille, sans presser. Elle est lisse, un peu mouillée. Il la glisse dans la poche. Elle est dans la poche. Tes mains sont au chaud ? Oui. Dans les poches. Ils rentrent dans la maison. La maison est tiède. La chaleur touche les joues de Victorino. Victorino retire le manteau rouge. Il le raccroche au crochet. Le crochet fait un petit bruit. Le manteau est à sa place. Je sors la feuille. Il prend la feuille dans la poche. Il la pose dans le bol blanc. Comme sur la vitre, maman ! Sur la feuille, un trait brille. Le &lt;emphasis level="moderate"&gt;trait de vitre&lt;/emphasis&gt; est sur la feuille. Tu le vois, sur ta feuille ? Oui. C'est ma feuille rouge. Le bol blanc garde la feuille. Le trait de vitre dore, mince.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Victorino ramasse la feuille, sans presser. Elle est lisse, un peu mouillée. Il la glisse dans la poche. Elle est dans la poche. Tes mains sont au chaud ? Oui. Dans les poches. Ils rentrent dans la maison. La maison est tiède. La chaleur touche les joues de Victorino. Victorino retire le manteau rouge. Il le raccroche au crochet. Le crochet fait un petit bruit. Le manteau est à sa place. Je sors la feuille. Il prend la feuille dans la poche. Il la pose dans le bol blanc. Comme sur la vitre, maman ! Sur la feuille, un trait brille. Le &lt;emphasis&gt;trait de vitre&lt;/emphasis&gt; est sur la feuille. Tu le vois, sur ta feuille ? Oui. C'est ma feuille rouge. Le bol blanc garde la feuille. Le trait de vitre dore, mince.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2026,7 +2062,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2034,7 +2070,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2046,12 +2082,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2060,17 +2096,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>trait de vitre</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2079,11 +2119,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2092,27 +2132,57 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=le_trait_de_vitre_est_sur_la_feuille; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai mis la feuille dans le bol.
-enfant-m|J'avais le manteau.
-maman|Bravo, Victorino.
-narrateur|Le bol blanc brille encore.</t>
+          <t>narrateur|Victorino ramasse la feuille, sans presser.
+narrateur|Elle est lisse, un peu mouillée.
+narrateur|Il la glisse dans la poche.
+enfant-m|Elle est dans la poche.
+maman|Tes mains sont au chaud ?
+enfant-m|Oui.
+enfant-m|Dans les poches.
+narrateur|Ils rentrent dans la maison.
+narrateur|La maison est tiède.
+narrateur|La chaleur touche les joues de Victorino.
+narrateur|Victorino retire le manteau rouge.
+narrateur|Il le raccroche au crochet.
+narrateur|Le crochet fait un petit bruit.
+narrateur|Le manteau est à sa place.
+enfant-m|Je sors la feuille.
+narrateur|Il prend la feuille dans la poche.
+narrateur|Il la pose dans le bol blanc.
+enfant-m|Comme sur la vitre, maman !
+narrateur|Sur la feuille, un trait brille.
+narrateur|Le trait de vitre est sur la feuille.
+maman|Tu le vois, sur ta feuille ?
+enfant-m|Oui.
+enfant-m|C'est ma feuille rouge.
+narrateur|Le bol blanc garde la feuille.
+narrateur|Le trait de vitre dore, mince.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>bol,feuille</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2225,6 +2295,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>